<commit_message>
Committing & pushing for backup purposes
</commit_message>
<xml_diff>
--- a/Amoritization.xlsx
+++ b/Amoritization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008F7A4B-86B6-4F9C-8BD1-AD4E6EE749B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCADC871-E717-4DED-8A42-FC90AC248F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4170" yWindow="1380" windowWidth="28800" windowHeight="15345" xr2:uid="{AE14A5DA-5418-4CB2-B16F-47804216F2DB}"/>
+    <workbookView xWindow="39285" yWindow="1500" windowWidth="33285" windowHeight="16605" xr2:uid="{AE14A5DA-5418-4CB2-B16F-47804216F2DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1219,18 +1219,18 @@
         <f>G13-B2</f>
         <v>2201.9003994796713</v>
       </c>
-      <c r="J13" s="29">
+      <c r="J13" s="20">
         <v>32</v>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="21">
         <f>K12*(1+C2)</f>
         <v>13749.406785310975</v>
       </c>
-      <c r="L13" s="30">
+      <c r="L13" s="21">
         <f>K12*C2</f>
         <v>136.13274044862351</v>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="22">
         <f>K13-B2</f>
         <v>3749.4067853109755</v>
       </c>

</xml_diff>